<commit_message>
Fixed issue when copying rows/columns where the format is not always preserved.
</commit_message>
<xml_diff>
--- a/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/CopyingRowsAndColumns.xlsx
+++ b/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/CopyingRowsAndColumns.xlsx
@@ -576,7 +576,7 @@
       <x:c r="A1" s="1" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+      <x:c r="B1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
@@ -596,15 +596,6 @@
       <x:c r="B2" s="0" t="s"/>
       <x:c r="D2" s="0" t="s"/>
       <x:c r="F2" s="0" t="s"/>
-    </x:row>
-    <x:row r="3" spans="1:6">
-      <x:c r="B3" s="0" t="s"/>
-    </x:row>
-    <x:row r="4" spans="1:6">
-      <x:c r="B4" s="0" t="s"/>
-    </x:row>
-    <x:row r="5" spans="1:6">
-      <x:c r="B5" s="0" t="s"/>
     </x:row>
     <x:row r="6" spans="1:6">
       <x:c r="B6" s="0" t="s"/>

</xml_diff>